<commit_message>
feat: update calibration projector and workflow tooling
</commit_message>
<xml_diff>
--- a/Documents/采购单/20250006-3D视觉系统研发电气技术变更单_20260417.xlsx
+++ b/Documents/采购单/20250006-3D视觉系统研发电气技术变更单_20260417.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17800"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="技术变更通知单" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="132">
   <si>
     <t>0006_OP010 3D视觉系统V1.0研发 技术变更单</t>
   </si>
@@ -333,6 +333,28 @@
   </si>
   <si>
     <t>https://item.taobao.com/item.htm?from=cart&amp;id=631926212362&amp;mi_id=0000bzHlHXa4uvlUHLf9ZtEfGxnpirVSI57DzlDFMP53KhE&amp;skuId=5083632269169&amp;spm=a1z0d.6639537%2F202410.item.d631926212362.1b1d7484WJK0rq&amp;upStreamPrice=21100</t>
+  </si>
+  <si>
+    <t>0006_OP010_063</t>
+  </si>
+  <si>
+    <t>名称：偏振片  数量2个
+型号：M27mm*P0.5线偏振镜
+料号 9980000715935</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?abbucket=3&amp;id=667339807480&amp;mi_id=0000dRsHVRlq1cSIGUEo5_RB84aZS5YqLsiYltRvVYr1xGE&amp;ns=1&amp;priceTId=2147825a17841630698231271e0f38&amp;skuId=5041628658578&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%22570948bb83f52a025bfa9b4f4968a9db%22%7D&amp;xxc=taobaoSearch</t>
+  </si>
+  <si>
+    <t>0006_OP010_064</t>
+  </si>
+  <si>
+    <t>名称：标定板  数量1个
+型号：11*11 圆点标定板
+料号 9980000715938</t>
+  </si>
+  <si>
+    <t>https://dfilm.taobao.com/shop/view_shop.htm?shop_id=423724622&amp;spm=a21m98.27004841</t>
   </si>
   <si>
     <t>项目名称</t>
@@ -490,7 +512,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="000000"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="35">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,18 +564,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -584,7 +594,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="14"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -1011,6 +1039,32 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -1052,19 +1106,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -1076,7 +1117,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -1106,21 +1149,6 @@
         <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1239,137 +1267,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1386,11 +1414,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1403,52 +1431,85 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1456,107 +1517,77 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -4944,15 +4975,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>335280</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>75565</xdr:rowOff>
+      <xdr:colOff>307340</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>61595</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>614680</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>478155</xdr:rowOff>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>464185</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -4961,7 +4992,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1021080" y="14535785"/>
+          <a:off x="993140" y="15144115"/>
           <a:ext cx="279400" cy="402590"/>
         </a:xfrm>
         <a:prstGeom prst="triangle">
@@ -5128,6 +5159,338 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1021715" y="13922375"/>
+          <a:ext cx="279400" cy="402590"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-CN">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="en-US" altLang="zh-CN" sz="1100">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>339090</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>93980</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>618490</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>496570</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="等腰三角形 9"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1024890" y="14554200"/>
+          <a:ext cx="279400" cy="402590"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:srgbClr val="FFFFFF"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
+        <a:lstStyle>
+          <a:defPPr>
+            <a:defRPr lang="zh-CN">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:defPPr>
+          <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="en-US" altLang="zh-CN" sz="1100">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>307340</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>61595</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>464185</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="等腰三角形 10"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="993140" y="15766415"/>
           <a:ext cx="279400" cy="402590"/>
         </a:xfrm>
         <a:prstGeom prst="triangle">
@@ -5563,7 +5926,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N50"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="12.0833333333333" customWidth="1"/>
     <col min="3" max="6" width="12.75" customWidth="1"/>
@@ -5609,1214 +5972,1238 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
-      <c r="M2" s="43" t="s">
+      <c r="M2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="44"/>
+      <c r="N2" s="13"/>
     </row>
     <row r="3" s="8" customFormat="1" ht="41.15" customHeight="1" spans="1:14">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="17"/>
+      <c r="E3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16" t="s">
+      <c r="F3" s="17"/>
+      <c r="G3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="14" t="s">
+      <c r="H3" s="17"/>
+      <c r="I3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="15"/>
-      <c r="K3" s="45" t="s">
+      <c r="J3" s="17"/>
+      <c r="K3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="45"/>
-      <c r="M3" s="46" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="47"/>
+      <c r="N3" s="21"/>
     </row>
     <row r="4" ht="20.15" customHeight="1" spans="1:14">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="18" t="s">
+      <c r="D4" s="24"/>
+      <c r="E4" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="19"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="18" t="s">
+      <c r="F4" s="24"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="20"/>
-      <c r="J4" s="21" t="s">
+      <c r="I4" s="25"/>
+      <c r="J4" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21" t="s">
+      <c r="K4" s="26"/>
+      <c r="L4" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21" t="s">
+      <c r="M4" s="26"/>
+      <c r="N4" s="26" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="49" customHeight="1" spans="1:14">
-      <c r="A5" s="21">
+      <c r="A5" s="26">
         <v>1</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="27">
         <v>1</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="26" t="s">
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="48"/>
-      <c r="J5" s="21" t="s">
+      <c r="I5" s="32"/>
+      <c r="J5" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="21"/>
-      <c r="L5" s="49">
+      <c r="K5" s="26"/>
+      <c r="L5" s="33">
         <v>46080</v>
       </c>
-      <c r="M5" s="20"/>
-      <c r="N5" s="50" t="s">
+      <c r="M5" s="25"/>
+      <c r="N5" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" ht="49" customHeight="1" spans="1:14">
-      <c r="A6" s="21">
+      <c r="A6" s="26">
         <v>2</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="27">
         <v>1</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26" t="s">
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="48"/>
-      <c r="J6" s="21" t="s">
+      <c r="I6" s="32"/>
+      <c r="J6" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="21"/>
-      <c r="L6" s="49">
+      <c r="K6" s="26"/>
+      <c r="L6" s="33">
         <v>46080</v>
       </c>
-      <c r="M6" s="20"/>
-      <c r="N6" s="51" t="s">
+      <c r="M6" s="25"/>
+      <c r="N6" s="35" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" ht="49" customHeight="1" spans="1:14">
-      <c r="A7" s="21">
+      <c r="A7" s="26">
         <v>3</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="36">
         <v>1</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26" t="s">
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="21" t="s">
+      <c r="I7" s="32"/>
+      <c r="J7" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="21"/>
-      <c r="L7" s="49">
+      <c r="K7" s="26"/>
+      <c r="L7" s="33">
         <v>46080</v>
       </c>
-      <c r="M7" s="20"/>
-      <c r="N7" s="51" t="s">
+      <c r="M7" s="25"/>
+      <c r="N7" s="35" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" ht="49" customHeight="1" spans="1:14">
-      <c r="A8" s="21">
+      <c r="A8" s="26">
         <v>4</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="36">
         <v>1</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26" t="s">
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="48"/>
-      <c r="J8" s="21" t="s">
+      <c r="I8" s="32"/>
+      <c r="J8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="21"/>
-      <c r="L8" s="49">
+      <c r="K8" s="26"/>
+      <c r="L8" s="33">
         <v>46080</v>
       </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="52" t="s">
+      <c r="M8" s="25"/>
+      <c r="N8" s="37" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" ht="49" customHeight="1" spans="1:14">
-      <c r="A9" s="21">
+      <c r="A9" s="26">
         <v>5</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="36">
         <v>1</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26" t="s">
+      <c r="D9" s="29"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="48"/>
-      <c r="J9" s="21" t="s">
+      <c r="I9" s="32"/>
+      <c r="J9" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="21"/>
-      <c r="L9" s="49">
+      <c r="K9" s="26"/>
+      <c r="L9" s="33">
         <v>46080</v>
       </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="53" t="s">
+      <c r="M9" s="25"/>
+      <c r="N9" s="38" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" ht="49" customHeight="1" spans="1:14">
-      <c r="A10" s="21">
+      <c r="A10" s="26">
         <v>6</v>
       </c>
-      <c r="B10" s="27">
+      <c r="B10" s="36">
         <v>1</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26" t="s">
+      <c r="D10" s="29"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="48" t="s">
+      <c r="I10" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="21"/>
-      <c r="L10" s="49">
+      <c r="K10" s="26"/>
+      <c r="L10" s="33">
         <v>46080</v>
       </c>
-      <c r="M10" s="20"/>
-      <c r="N10" s="53">
+      <c r="M10" s="25"/>
+      <c r="N10" s="38">
         <v>18960739823</v>
       </c>
     </row>
     <row r="11" ht="49" customHeight="1" spans="1:14">
-      <c r="A11" s="21">
+      <c r="A11" s="26">
         <v>7</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="36">
         <v>1</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26" t="s">
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="I11" s="48" t="s">
+      <c r="I11" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="21"/>
-      <c r="L11" s="49">
+      <c r="K11" s="26"/>
+      <c r="L11" s="33">
         <v>46080</v>
       </c>
-      <c r="M11" s="20"/>
-      <c r="N11" s="53">
+      <c r="M11" s="25"/>
+      <c r="N11" s="38">
         <v>18668172091</v>
       </c>
     </row>
     <row r="12" ht="49" customHeight="1" spans="1:14">
-      <c r="A12" s="21">
+      <c r="A12" s="26">
         <v>8</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="36">
         <v>1</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26" t="s">
+      <c r="D12" s="29"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="48" t="s">
+      <c r="I12" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="21"/>
-      <c r="L12" s="49">
+      <c r="K12" s="26"/>
+      <c r="L12" s="33">
         <v>46080</v>
       </c>
-      <c r="M12" s="20"/>
-      <c r="N12" s="53"/>
+      <c r="M12" s="25"/>
+      <c r="N12" s="38"/>
     </row>
     <row r="13" ht="49" customHeight="1" spans="1:14">
-      <c r="A13" s="21">
+      <c r="A13" s="26">
         <v>9</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="36">
         <v>1</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="26" t="s">
+      <c r="D13" s="29"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="I13" s="48" t="s">
+      <c r="I13" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="J13" s="21" t="s">
+      <c r="J13" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="21"/>
-      <c r="L13" s="49">
+      <c r="K13" s="26"/>
+      <c r="L13" s="33">
         <v>46080</v>
       </c>
-      <c r="M13" s="20"/>
-      <c r="N13" s="53"/>
+      <c r="M13" s="25"/>
+      <c r="N13" s="38"/>
     </row>
     <row r="14" ht="49" customHeight="1" spans="1:14">
-      <c r="A14" s="21">
+      <c r="A14" s="26">
         <v>10</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="36">
         <v>1</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="26" t="s">
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="48" t="s">
+      <c r="I14" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="J14" s="21" t="s">
+      <c r="J14" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K14" s="21"/>
-      <c r="L14" s="49">
+      <c r="K14" s="26"/>
+      <c r="L14" s="33">
         <v>46080</v>
       </c>
-      <c r="M14" s="20"/>
-      <c r="N14" s="53">
+      <c r="M14" s="25"/>
+      <c r="N14" s="38">
         <v>13539986755</v>
       </c>
     </row>
     <row r="15" ht="49" customHeight="1" spans="1:14">
-      <c r="A15" s="21">
+      <c r="A15" s="26">
         <v>11</v>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="36">
         <v>1</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="26" t="s">
+      <c r="D15" s="29"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="I15" s="48" t="s">
+      <c r="I15" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="J15" s="21" t="s">
+      <c r="J15" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="21"/>
-      <c r="L15" s="49">
+      <c r="K15" s="26"/>
+      <c r="L15" s="33">
         <v>46080</v>
       </c>
-      <c r="M15" s="20"/>
-      <c r="N15" s="53" t="s">
+      <c r="M15" s="25"/>
+      <c r="N15" s="38" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="16" ht="49" customHeight="1" spans="1:14">
-      <c r="A16" s="21">
+      <c r="A16" s="26">
         <v>12</v>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="36">
         <v>1</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="26" t="s">
+      <c r="D16" s="29"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="I16" s="48" t="s">
+      <c r="I16" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="21" t="s">
+      <c r="J16" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K16" s="21"/>
-      <c r="L16" s="49">
+      <c r="K16" s="26"/>
+      <c r="L16" s="33">
         <v>46080</v>
       </c>
-      <c r="M16" s="20"/>
-      <c r="N16" s="53" t="s">
+      <c r="M16" s="25"/>
+      <c r="N16" s="38" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="17" ht="49" customHeight="1" spans="1:14">
-      <c r="A17" s="21">
+      <c r="A17" s="26">
         <v>13</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="36">
         <v>1</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="26" t="s">
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="I17" s="48" t="s">
+      <c r="I17" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="J17" s="21" t="s">
+      <c r="J17" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K17" s="21"/>
-      <c r="L17" s="49">
+      <c r="K17" s="26"/>
+      <c r="L17" s="33">
         <v>46080</v>
       </c>
-      <c r="M17" s="20"/>
-      <c r="N17" s="53" t="s">
+      <c r="M17" s="25"/>
+      <c r="N17" s="38" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="18" ht="49" customHeight="1" spans="1:14">
-      <c r="A18" s="21">
+      <c r="A18" s="26">
         <v>14</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="36">
         <v>1</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26" t="s">
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="48" t="s">
+      <c r="I18" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="J18" s="21" t="s">
+      <c r="J18" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="21"/>
-      <c r="L18" s="49">
+      <c r="K18" s="26"/>
+      <c r="L18" s="33">
         <v>46080</v>
       </c>
-      <c r="M18" s="20"/>
-      <c r="N18" s="53" t="s">
+      <c r="M18" s="25"/>
+      <c r="N18" s="38" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" ht="49" customHeight="1" spans="1:14">
-      <c r="A19" s="21">
+      <c r="A19" s="26">
         <v>15</v>
       </c>
-      <c r="B19" s="27">
+      <c r="B19" s="36">
         <v>1</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="26" t="s">
+      <c r="D19" s="29"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="48" t="s">
+      <c r="I19" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="21" t="s">
+      <c r="J19" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K19" s="21"/>
-      <c r="L19" s="49">
+      <c r="K19" s="26"/>
+      <c r="L19" s="33">
         <v>46080</v>
       </c>
-      <c r="M19" s="20"/>
-      <c r="N19" s="53" t="s">
+      <c r="M19" s="25"/>
+      <c r="N19" s="38" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="20" ht="49" customHeight="1" spans="1:14">
-      <c r="A20" s="21">
+      <c r="A20" s="26">
         <v>16</v>
       </c>
-      <c r="B20" s="27">
+      <c r="B20" s="36">
         <v>1</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="26" t="s">
+      <c r="D20" s="29"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="I20" s="48" t="s">
+      <c r="I20" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="J20" s="21" t="s">
+      <c r="J20" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K20" s="21"/>
-      <c r="L20" s="49">
+      <c r="K20" s="26"/>
+      <c r="L20" s="33">
         <v>46080</v>
       </c>
-      <c r="M20" s="20"/>
-      <c r="N20" s="53" t="s">
+      <c r="M20" s="25"/>
+      <c r="N20" s="38" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="21" ht="49" customHeight="1" spans="1:14">
-      <c r="A21" s="21">
+      <c r="A21" s="26">
         <v>17</v>
       </c>
-      <c r="B21" s="27">
+      <c r="B21" s="36">
         <v>1</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="26" t="s">
+      <c r="D21" s="29"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="I21" s="48" t="s">
+      <c r="I21" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="J21" s="21" t="s">
+      <c r="J21" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="49">
+      <c r="K21" s="26"/>
+      <c r="L21" s="33">
         <v>46080</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="53" t="s">
+      <c r="M21" s="25"/>
+      <c r="N21" s="38" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="22" ht="49" customHeight="1" spans="1:14">
-      <c r="A22" s="21">
+      <c r="A22" s="26">
         <v>18</v>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="36">
         <v>1</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="24"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="26" t="s">
+      <c r="D22" s="29"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="I22" s="48" t="s">
+      <c r="I22" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="J22" s="21" t="s">
+      <c r="J22" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K22" s="21"/>
-      <c r="L22" s="49">
+      <c r="K22" s="26"/>
+      <c r="L22" s="33">
         <v>46080</v>
       </c>
-      <c r="M22" s="20"/>
-      <c r="N22" s="53" t="s">
+      <c r="M22" s="25"/>
+      <c r="N22" s="38" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="23" ht="49" customHeight="1" spans="1:14">
-      <c r="A23" s="21">
+      <c r="A23" s="26">
         <v>19</v>
       </c>
-      <c r="B23" s="27">
+      <c r="B23" s="36">
         <v>1</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="26" t="s">
+      <c r="D23" s="29"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="J23" s="21" t="s">
+      <c r="J23" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="21"/>
-      <c r="L23" s="49">
+      <c r="K23" s="26"/>
+      <c r="L23" s="33">
         <v>46080</v>
       </c>
-      <c r="M23" s="20"/>
-      <c r="N23" s="53" t="s">
+      <c r="M23" s="25"/>
+      <c r="N23" s="38" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="24" ht="49" customHeight="1" spans="1:14">
-      <c r="A24" s="21">
+      <c r="A24" s="26">
         <v>20</v>
       </c>
-      <c r="B24" s="28">
+      <c r="B24" s="39">
         <v>2</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="25" t="s">
+      <c r="D24" s="40"/>
+      <c r="E24" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="26" t="s">
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="I24" s="48"/>
-      <c r="J24" s="21" t="s">
+      <c r="I24" s="32"/>
+      <c r="J24" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="K24" s="21"/>
-      <c r="L24" s="49">
+      <c r="K24" s="26"/>
+      <c r="L24" s="33">
         <v>46129</v>
       </c>
-      <c r="M24" s="20"/>
-      <c r="N24" s="54" t="s">
+      <c r="M24" s="25"/>
+      <c r="N24" s="41" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="25" ht="49" customHeight="1" spans="1:14">
-      <c r="A25" s="21">
+      <c r="A25" s="26">
         <v>21</v>
       </c>
-      <c r="B25" s="28">
+      <c r="B25" s="39">
         <v>2</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="25" t="s">
+      <c r="D25" s="40"/>
+      <c r="E25" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="26" t="s">
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="I25" s="48"/>
-      <c r="J25" s="21" t="s">
+      <c r="I25" s="32"/>
+      <c r="J25" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="K25" s="21"/>
-      <c r="L25" s="49">
+      <c r="K25" s="26"/>
+      <c r="L25" s="33">
         <v>46129</v>
       </c>
-      <c r="M25" s="20"/>
-      <c r="N25" s="55"/>
+      <c r="M25" s="25"/>
+      <c r="N25" s="42"/>
     </row>
     <row r="26" ht="49" customHeight="1" spans="1:14">
-      <c r="A26" s="21">
+      <c r="A26" s="26">
         <v>22</v>
       </c>
-      <c r="B26" s="28">
+      <c r="B26" s="39">
         <v>2</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="29"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="26" t="s">
+      <c r="D26" s="40"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="I26" s="48"/>
-      <c r="J26" s="21" t="s">
+      <c r="I26" s="32"/>
+      <c r="J26" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="K26" s="21"/>
-      <c r="L26" s="49">
+      <c r="K26" s="26"/>
+      <c r="L26" s="33">
         <v>46129</v>
       </c>
-      <c r="M26" s="20"/>
-      <c r="N26" s="56" t="s">
+      <c r="M26" s="25"/>
+      <c r="N26" s="43" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="27" ht="49" customHeight="1" spans="1:14">
-      <c r="A27" s="21">
+      <c r="A27" s="26">
         <v>23</v>
       </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="49"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="54"/>
+      <c r="B27" s="39">
+        <v>3</v>
+      </c>
+      <c r="C27" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="40"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="I27" s="32"/>
+      <c r="J27" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K27" s="26"/>
+      <c r="L27" s="33">
+        <v>46223</v>
+      </c>
+      <c r="M27" s="25"/>
+      <c r="N27" s="44" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="28" ht="49" customHeight="1" spans="1:14">
-      <c r="A28" s="21">
+      <c r="A28" s="26">
         <v>24</v>
       </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="48"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="49"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="54"/>
+      <c r="B28" s="39">
+        <v>3</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="40"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="I28" s="32"/>
+      <c r="J28" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K28" s="26"/>
+      <c r="L28" s="33">
+        <v>46223</v>
+      </c>
+      <c r="M28" s="25"/>
+      <c r="N28" s="44" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="29" ht="49" customHeight="1" spans="1:14">
-      <c r="A29" s="21">
+      <c r="A29" s="26">
         <v>25</v>
       </c>
-      <c r="B29" s="30"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="48"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="49"/>
-      <c r="M29" s="20"/>
-      <c r="N29" s="55"/>
+      <c r="B29" s="45"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="40"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="25"/>
+      <c r="N29" s="42"/>
     </row>
     <row r="30" ht="49" customHeight="1" spans="1:14">
-      <c r="A30" s="21">
+      <c r="A30" s="26">
         <v>26</v>
       </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="48"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="49"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="54"/>
+      <c r="B30" s="45"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="25"/>
+      <c r="N30" s="41"/>
     </row>
     <row r="31" ht="49" customHeight="1" spans="1:14">
-      <c r="A31" s="21">
+      <c r="A31" s="26">
         <v>27</v>
       </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="48"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="49"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="54"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="25"/>
+      <c r="N31" s="41"/>
     </row>
     <row r="32" ht="49" customHeight="1" spans="1:14">
-      <c r="A32" s="21">
+      <c r="A32" s="26">
         <v>28</v>
       </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="48"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="49"/>
-      <c r="M32" s="20"/>
-      <c r="N32" s="54"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="40"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="25"/>
+      <c r="N32" s="41"/>
     </row>
     <row r="33" ht="49" customHeight="1" spans="1:14">
-      <c r="A33" s="21">
+      <c r="A33" s="26">
         <v>29</v>
       </c>
-      <c r="B33" s="30"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="48"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="49"/>
-      <c r="M33" s="20"/>
-      <c r="N33" s="54"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="25"/>
+      <c r="N33" s="41"/>
     </row>
     <row r="34" ht="49" customHeight="1" spans="1:14">
-      <c r="A34" s="21">
+      <c r="A34" s="26">
         <v>30</v>
       </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="48"/>
-      <c r="J34" s="21"/>
-      <c r="K34" s="21"/>
-      <c r="L34" s="49"/>
-      <c r="M34" s="20"/>
-      <c r="N34" s="54"/>
+      <c r="B34" s="45"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="25"/>
+      <c r="N34" s="41"/>
     </row>
     <row r="35" ht="49" customHeight="1" spans="1:14">
-      <c r="A35" s="21">
+      <c r="A35" s="26">
         <v>31</v>
       </c>
-      <c r="B35" s="30"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="48"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="21"/>
-      <c r="L35" s="49"/>
-      <c r="M35" s="20"/>
-      <c r="N35" s="54"/>
+      <c r="B35" s="45"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="33"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="41"/>
     </row>
     <row r="36" ht="49" customHeight="1" spans="1:14">
-      <c r="A36" s="21">
+      <c r="A36" s="26">
         <v>32</v>
       </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="48"/>
-      <c r="J36" s="21"/>
-      <c r="K36" s="21"/>
-      <c r="L36" s="49"/>
-      <c r="M36" s="20"/>
-      <c r="N36" s="54"/>
+      <c r="B36" s="45"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="33"/>
+      <c r="M36" s="25"/>
+      <c r="N36" s="41"/>
     </row>
     <row r="37" ht="49" customHeight="1" spans="1:14">
-      <c r="A37" s="21">
+      <c r="A37" s="26">
         <v>33</v>
       </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="48"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
-      <c r="L37" s="49"/>
-      <c r="M37" s="20"/>
-      <c r="N37" s="54"/>
+      <c r="B37" s="45"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="26"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="33"/>
+      <c r="M37" s="25"/>
+      <c r="N37" s="41"/>
     </row>
     <row r="38" ht="49" customHeight="1" spans="1:14">
-      <c r="A38" s="21">
+      <c r="A38" s="26">
         <v>34</v>
       </c>
-      <c r="B38" s="30"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="48"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="21"/>
-      <c r="L38" s="49"/>
-      <c r="M38" s="20"/>
-      <c r="N38" s="54"/>
+      <c r="B38" s="45"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="26"/>
+      <c r="K38" s="26"/>
+      <c r="L38" s="33"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="41"/>
     </row>
     <row r="39" ht="49" customHeight="1" spans="1:14">
-      <c r="A39" s="21">
+      <c r="A39" s="26">
         <v>35</v>
       </c>
-      <c r="B39" s="30"/>
-      <c r="C39" s="29"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="48"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="49"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="55"/>
+      <c r="B39" s="45"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="31"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="26"/>
+      <c r="K39" s="26"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="25"/>
+      <c r="N39" s="42"/>
     </row>
     <row r="40" ht="49" customHeight="1" spans="1:14">
-      <c r="A40" s="21">
+      <c r="A40" s="26">
         <v>36</v>
       </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="25"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="48"/>
-      <c r="J40" s="21"/>
-      <c r="K40" s="21"/>
-      <c r="L40" s="57"/>
-      <c r="M40" s="58"/>
-      <c r="N40" s="55"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="26"/>
+      <c r="K40" s="26"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="47"/>
+      <c r="N40" s="42"/>
     </row>
     <row r="41" ht="49" customHeight="1" spans="1:14">
-      <c r="A41" s="21">
+      <c r="A41" s="26">
         <v>37</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="25"/>
-      <c r="G41" s="25"/>
-      <c r="H41" s="31"/>
+      <c r="B41" s="39"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="30"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="30"/>
+      <c r="H41" s="48"/>
       <c r="I41" s="9"/>
-      <c r="J41" s="18"/>
-      <c r="K41" s="20"/>
-      <c r="L41" s="57"/>
-      <c r="M41" s="58"/>
-      <c r="N41" s="54"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="46"/>
+      <c r="M41" s="47"/>
+      <c r="N41" s="41"/>
     </row>
     <row r="42" ht="49" customHeight="1" spans="1:14">
-      <c r="A42" s="21">
+      <c r="A42" s="26">
         <v>38</v>
       </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="25"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="48"/>
-      <c r="J42" s="21"/>
-      <c r="K42" s="21"/>
-      <c r="L42" s="57"/>
-      <c r="M42" s="58"/>
-      <c r="N42" s="54"/>
+      <c r="B42" s="39"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="30"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="26"/>
+      <c r="K42" s="26"/>
+      <c r="L42" s="46"/>
+      <c r="M42" s="47"/>
+      <c r="N42" s="41"/>
     </row>
     <row r="43" ht="49" customHeight="1" spans="1:14">
-      <c r="A43" s="21">
+      <c r="A43" s="26">
         <v>39</v>
       </c>
-      <c r="B43" s="22"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25"/>
-      <c r="G43" s="25"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="48"/>
-      <c r="J43" s="21"/>
-      <c r="K43" s="21"/>
-      <c r="L43" s="57"/>
-      <c r="M43" s="58"/>
-      <c r="N43" s="54"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="31"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="26"/>
+      <c r="K43" s="26"/>
+      <c r="L43" s="46"/>
+      <c r="M43" s="47"/>
+      <c r="N43" s="41"/>
     </row>
     <row r="44" ht="49" customHeight="1" spans="1:14">
-      <c r="A44" s="21">
+      <c r="A44" s="26">
         <v>40</v>
       </c>
-      <c r="B44" s="22"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25"/>
-      <c r="G44" s="25"/>
-      <c r="H44" s="26"/>
-      <c r="I44" s="48"/>
-      <c r="J44" s="21"/>
-      <c r="K44" s="21"/>
-      <c r="L44" s="57"/>
-      <c r="M44" s="58"/>
-      <c r="N44" s="54"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="52"/>
+      <c r="E44" s="30"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="26"/>
+      <c r="K44" s="26"/>
+      <c r="L44" s="46"/>
+      <c r="M44" s="47"/>
+      <c r="N44" s="41"/>
     </row>
     <row r="45" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A45" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="37"/>
-      <c r="C45" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="D45" s="38"/>
-      <c r="E45" s="38"/>
-      <c r="F45" s="38"/>
-      <c r="G45" s="38"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="59" t="s">
-        <v>80</v>
-      </c>
-      <c r="J45" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="K45" s="37"/>
-      <c r="L45" s="37"/>
-      <c r="M45" s="37"/>
-      <c r="N45" s="60"/>
+      <c r="A45" s="53" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" s="54"/>
+      <c r="C45" s="55" t="s">
+        <v>85</v>
+      </c>
+      <c r="D45" s="55"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="55"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="56" t="s">
+        <v>86</v>
+      </c>
+      <c r="J45" s="57" t="s">
+        <v>87</v>
+      </c>
+      <c r="K45" s="54"/>
+      <c r="L45" s="54"/>
+      <c r="M45" s="54"/>
+      <c r="N45" s="58"/>
     </row>
     <row r="46" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A46" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B46" s="37"/>
-      <c r="C46" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="38"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="59" t="s">
-        <v>83</v>
-      </c>
-      <c r="J46" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="K46" s="37"/>
-      <c r="L46" s="37"/>
-      <c r="M46" s="37"/>
-      <c r="N46" s="60"/>
+      <c r="A46" s="57" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" s="54"/>
+      <c r="C46" s="55" t="s">
+        <v>85</v>
+      </c>
+      <c r="D46" s="55"/>
+      <c r="E46" s="55"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="55"/>
+      <c r="H46" s="55"/>
+      <c r="I46" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="J46" s="57" t="s">
+        <v>90</v>
+      </c>
+      <c r="K46" s="54"/>
+      <c r="L46" s="54"/>
+      <c r="M46" s="54"/>
+      <c r="N46" s="58"/>
     </row>
     <row r="47" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A47" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="B47" s="37"/>
-      <c r="C47" s="39"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="39"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="59" t="s">
-        <v>86</v>
-      </c>
-      <c r="J47" s="61"/>
-      <c r="K47" s="62"/>
-      <c r="L47" s="62"/>
-      <c r="M47" s="62"/>
-      <c r="N47" s="63"/>
+      <c r="A47" s="57" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="54"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="54"/>
+      <c r="E47" s="57"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="54"/>
+      <c r="I47" s="56" t="s">
+        <v>92</v>
+      </c>
+      <c r="J47" s="59"/>
+      <c r="K47" s="60"/>
+      <c r="L47" s="60"/>
+      <c r="M47" s="60"/>
+      <c r="N47" s="61"/>
     </row>
     <row r="48" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A48" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="B48" s="37"/>
-      <c r="C48" s="39" t="str">
+      <c r="A48" s="57" t="s">
+        <v>93</v>
+      </c>
+      <c r="B48" s="54"/>
+      <c r="C48" s="57" t="str">
         <f>LEFT(J45,7)&amp;RIGHT(J45,7)&amp;"-"&amp;C47</f>
         <v>T024-200250006-</v>
       </c>
-      <c r="D48" s="37"/>
-      <c r="E48" s="39"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="37"/>
-      <c r="I48" s="59" t="s">
-        <v>88</v>
-      </c>
-      <c r="J48" s="39" t="str">
+      <c r="D48" s="54"/>
+      <c r="E48" s="57"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="54"/>
+      <c r="H48" s="54"/>
+      <c r="I48" s="56" t="s">
+        <v>94</v>
+      </c>
+      <c r="J48" s="57" t="str">
         <f>LEFT(J46,4)&amp;RIGHT(J46,13)&amp;"-"&amp;J47</f>
         <v>T0240250006-01-01-</v>
       </c>
-      <c r="K48" s="37"/>
-      <c r="L48" s="37"/>
-      <c r="M48" s="37"/>
-      <c r="N48" s="60"/>
+      <c r="K48" s="54"/>
+      <c r="L48" s="54"/>
+      <c r="M48" s="54"/>
+      <c r="N48" s="58"/>
     </row>
     <row r="49" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A49" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="B49" s="40"/>
-      <c r="C49" s="40"/>
-      <c r="D49" s="40"/>
-      <c r="E49" s="40"/>
-      <c r="F49" s="41"/>
-      <c r="G49" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="H49" s="42"/>
-      <c r="I49" s="42"/>
-      <c r="J49" s="42"/>
-      <c r="K49" s="42"/>
-      <c r="L49" s="42"/>
-      <c r="M49" s="42"/>
-      <c r="N49" s="42"/>
+      <c r="A49" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" s="62"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="64" t="s">
+        <v>96</v>
+      </c>
+      <c r="H49" s="64"/>
+      <c r="I49" s="64"/>
+      <c r="J49" s="64"/>
+      <c r="K49" s="64"/>
+      <c r="L49" s="64"/>
+      <c r="M49" s="64"/>
+      <c r="N49" s="64"/>
     </row>
     <row r="50" ht="35.15" customHeight="1" spans="1:14">
-      <c r="A50" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="B50" s="40"/>
-      <c r="C50" s="40"/>
-      <c r="D50" s="40"/>
-      <c r="E50" s="40"/>
-      <c r="F50" s="41"/>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="42"/>
-      <c r="J50" s="42"/>
-      <c r="K50" s="42"/>
-      <c r="L50" s="42"/>
-      <c r="M50" s="42"/>
-      <c r="N50" s="42"/>
+      <c r="A50" s="53" t="s">
+        <v>97</v>
+      </c>
+      <c r="B50" s="62"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="62"/>
+      <c r="E50" s="62"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="64"/>
+      <c r="H50" s="64"/>
+      <c r="I50" s="64"/>
+      <c r="J50" s="64"/>
+      <c r="K50" s="64"/>
+      <c r="L50" s="64"/>
+      <c r="M50" s="64"/>
+      <c r="N50" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="223">
@@ -7060,7 +7447,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.707638888888889" right="0.707638888888889" top="0.747916666666667" bottom="0.275" header="0.313888888888889" footer="0.313888888888889"/>
-  <pageSetup paperSize="8" scale="54" orientation="portrait"/>
+  <pageSetup paperSize="8" scale="55" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;G&amp;C&amp;"宋体,常规"&amp;16浙 江 三 花 汽 车 零 部 件 有 限 公 司&amp;R第&amp;P页 共2页</oddHeader>
   </headerFooter>
@@ -7074,7 +7461,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="65.0833333333333" customWidth="1"/>
     <col min="2" max="2" width="12.6666666666667" customWidth="1"/>
@@ -7082,409 +7469,409 @@
     <col min="9" max="9" width="19.1666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" spans="1:9">
+    <row r="1" ht="42.75" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D1" s="3">
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" s="7">
+        <v>103</v>
+      </c>
+      <c r="I1" s="6">
         <v>9980000658009</v>
       </c>
     </row>
-    <row r="2" ht="42" spans="1:9">
+    <row r="2" ht="42.75" spans="1:9">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I2" s="7">
+        <v>108</v>
+      </c>
+      <c r="I2" s="6">
         <v>9980000658010</v>
       </c>
     </row>
-    <row r="3" ht="42" spans="1:9">
+    <row r="3" ht="42.75" spans="1:9">
       <c r="A3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D3" s="3">
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I3" s="7">
+        <v>112</v>
+      </c>
+      <c r="I3" s="6">
         <v>9980000658011</v>
       </c>
     </row>
-    <row r="4" ht="42" spans="1:9">
+    <row r="4" ht="42.75" spans="1:9">
       <c r="A4" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I4" s="7">
+        <v>112</v>
+      </c>
+      <c r="I4" s="6">
         <v>9980000658014</v>
       </c>
     </row>
-    <row r="5" ht="42" spans="1:9">
+    <row r="5" ht="42.75" spans="1:9">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I5" s="7">
+        <v>112</v>
+      </c>
+      <c r="I5" s="6">
         <v>9980000658016</v>
       </c>
     </row>
-    <row r="6" ht="42" spans="1:9">
+    <row r="6" ht="42.75" spans="1:9">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I6" s="7">
+        <v>112</v>
+      </c>
+      <c r="I6" s="6">
         <v>9980000658017</v>
       </c>
     </row>
-    <row r="7" ht="42" spans="1:9">
+    <row r="7" ht="42.75" spans="1:9">
       <c r="A7" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I7" s="7">
+        <v>112</v>
+      </c>
+      <c r="I7" s="6">
         <v>9980000658018</v>
       </c>
     </row>
-    <row r="8" ht="42" spans="1:9">
+    <row r="8" ht="42.75" spans="1:9">
       <c r="A8" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I8" s="7">
+        <v>112</v>
+      </c>
+      <c r="I8" s="6">
         <v>9980000658019</v>
       </c>
     </row>
-    <row r="9" ht="42" spans="1:9">
+    <row r="9" ht="42.75" spans="1:9">
       <c r="A9" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D9" s="3">
         <v>30</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I9" s="7">
+        <v>112</v>
+      </c>
+      <c r="I9" s="6">
         <v>9980000658021</v>
       </c>
     </row>
-    <row r="10" ht="42" spans="1:9">
+    <row r="10" ht="42.75" spans="1:9">
       <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D10" s="3">
         <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I10" s="7">
+        <v>112</v>
+      </c>
+      <c r="I10" s="6">
         <v>9980000658022</v>
       </c>
     </row>
-    <row r="11" ht="42" spans="1:9">
+    <row r="11" ht="42.75" spans="1:9">
       <c r="A11" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D11" s="3">
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I11" s="7">
+        <v>112</v>
+      </c>
+      <c r="I11" s="6">
         <v>9980000658023</v>
       </c>
     </row>
-    <row r="12" ht="42" spans="1:9">
+    <row r="12" ht="42.75" spans="1:9">
       <c r="A12" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C12" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D12" s="3">
         <v>50</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I12" s="7">
+        <v>112</v>
+      </c>
+      <c r="I12" s="6">
         <v>9980000658024</v>
       </c>
     </row>
-    <row r="13" ht="42" spans="1:9">
+    <row r="13" ht="42.75" spans="1:9">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D13" s="3">
         <v>4</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I13" s="7">
+        <v>112</v>
+      </c>
+      <c r="I13" s="6">
         <v>9980000658026</v>
       </c>
     </row>
-    <row r="14" ht="42" spans="1:9">
+    <row r="14" ht="42.75" spans="1:9">
       <c r="A14" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D14" s="3">
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>125</v>
+        <v>106</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>131</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I14" s="7">
+        <v>112</v>
+      </c>
+      <c r="I14" s="6">
         <v>9980000658030</v>
       </c>
     </row>

</xml_diff>